<commit_message>
Sprint 5: Epics 07, 08 & 09 Cash Flow Intelligence + Reports + NLP complete - 92 tearsheet PDFs, 75 unit tests
</commit_message>
<xml_diff>
--- a/output/screener_output.xlsx
+++ b/output/screener_output.xlsx
@@ -612,7 +612,7 @@
         <v>13.59</v>
       </c>
       <c r="T2" t="n">
-        <v>26.65</v>
+        <v>34.75</v>
       </c>
     </row>
     <row r="3">
@@ -677,7 +677,7 @@
         <v>18.59</v>
       </c>
       <c r="T3" t="n">
-        <v>27.43</v>
+        <v>31.45</v>
       </c>
     </row>
     <row r="4">
@@ -742,7 +742,7 @@
         <v>22.78</v>
       </c>
       <c r="T4" t="n">
-        <v>26.4</v>
+        <v>34.76</v>
       </c>
     </row>
     <row r="5">
@@ -807,7 +807,7 @@
         <v>9.41</v>
       </c>
       <c r="T5" t="n">
-        <v>29.07</v>
+        <v>22.23</v>
       </c>
     </row>
     <row r="6">
@@ -872,7 +872,7 @@
         <v>0.47</v>
       </c>
       <c r="T6" t="n">
-        <v>17.92</v>
+        <v>32.82</v>
       </c>
     </row>
     <row r="7">
@@ -937,7 +937,7 @@
         <v>0.57</v>
       </c>
       <c r="T7" t="n">
-        <v>28.07</v>
+        <v>24.79</v>
       </c>
     </row>
     <row r="8">
@@ -1002,7 +1002,7 @@
         <v>-2.18</v>
       </c>
       <c r="T8" t="n">
-        <v>31.74</v>
+        <v>34.52</v>
       </c>
     </row>
     <row r="9">
@@ -1067,7 +1067,7 @@
         <v>-5.42</v>
       </c>
       <c r="T9" t="n">
-        <v>15.47</v>
+        <v>23.47</v>
       </c>
     </row>
   </sheetData>
@@ -1081,7 +1081,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T16"/>
+  <dimension ref="A1:T11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1188,977 +1188,652 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>56</v>
+        <v>49</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>TECHM</t>
+          <t>HDFCLIFE</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>TECHM India Limited</t>
+          <t>HDFCLIFE India Limited</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Oil &amp; Gas</t>
+          <t>Automobile</t>
         </is>
       </c>
       <c r="E2" t="n">
-        <v>65.53</v>
+        <v>67.59</v>
       </c>
       <c r="F2" t="n">
-        <v>199.87</v>
+        <v>259.26</v>
       </c>
       <c r="G2" t="n">
-        <v>268.93</v>
+        <v>384.41</v>
       </c>
       <c r="H2" t="n">
-        <v>12.84</v>
+        <v>9.56</v>
       </c>
       <c r="I2" s="2" t="n">
-        <v>0.4</v>
+        <v>0.39</v>
       </c>
       <c r="J2" t="n">
-        <v>8.039999999999999</v>
+        <v>6.58</v>
       </c>
       <c r="L2" t="n">
-        <v>1625.7</v>
+        <v>1324.15</v>
       </c>
       <c r="M2" t="n">
-        <v>0.24</v>
+        <v>0.19</v>
       </c>
       <c r="N2" t="n">
-        <v>2438.56</v>
+        <v>1986.22</v>
       </c>
       <c r="O2" t="n">
-        <v>4.59</v>
+        <v>4.58</v>
       </c>
       <c r="P2" t="n">
-        <v>205.65</v>
+        <v>155.78</v>
       </c>
       <c r="Q2" t="n">
         <v>10</v>
       </c>
       <c r="R2" t="n">
-        <v>12.99</v>
+        <v>16.36</v>
       </c>
       <c r="S2" t="n">
-        <v>12.99</v>
+        <v>16.36</v>
       </c>
       <c r="T2" t="n">
-        <v>16.03</v>
+        <v>17.28</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>7</v>
+        <v>75</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>ITC</t>
+          <t>MAXHEALTH</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>ITC India Limited</t>
+          <t>MAXHEALTH India Limited</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Power</t>
+          <t>Consumer Goods</t>
         </is>
       </c>
       <c r="E3" t="n">
-        <v>63.53</v>
+        <v>54.41</v>
       </c>
       <c r="F3" t="n">
-        <v>36.47</v>
+        <v>61.14</v>
       </c>
       <c r="G3" t="n">
-        <v>46.11</v>
+        <v>81.62</v>
       </c>
       <c r="H3" t="n">
-        <v>16.14</v>
+        <v>13.11</v>
       </c>
       <c r="I3" s="2" t="n">
         <v>0.4</v>
       </c>
       <c r="J3" t="n">
-        <v>9.51</v>
+        <v>8.16</v>
       </c>
       <c r="L3" t="n">
-        <v>1922.24</v>
+        <v>1937.82</v>
       </c>
       <c r="M3" t="n">
-        <v>1.24</v>
+        <v>0.22</v>
       </c>
       <c r="N3" t="n">
-        <v>2883.37</v>
+        <v>2906.72</v>
       </c>
       <c r="O3" t="n">
-        <v>20.22</v>
+        <v>5.99</v>
       </c>
       <c r="P3" t="n">
-        <v>57.85</v>
+        <v>188.79</v>
       </c>
       <c r="Q3" t="n">
         <v>10</v>
       </c>
       <c r="R3" t="n">
-        <v>31.75</v>
+        <v>25.42</v>
       </c>
       <c r="S3" t="n">
-        <v>31.76</v>
+        <v>25.43</v>
       </c>
       <c r="T3" t="n">
-        <v>19.6</v>
+        <v>17.69</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>71</v>
+        <v>68</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>JIOFIN</t>
+          <t>SRF</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>JIOFIN India Limited</t>
+          <t>SRF India Limited</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Construction</t>
+          <t>Metals</t>
         </is>
       </c>
       <c r="E4" t="n">
-        <v>55.62</v>
+        <v>45.83</v>
       </c>
       <c r="F4" t="n">
-        <v>127.37</v>
+        <v>119.91</v>
       </c>
       <c r="G4" t="n">
-        <v>183.53</v>
+        <v>221.34</v>
       </c>
       <c r="H4" t="n">
-        <v>10.3</v>
+        <v>5.66</v>
       </c>
       <c r="I4" s="2" t="n">
-        <v>0.4</v>
+        <v>0.39</v>
       </c>
       <c r="J4" t="n">
-        <v>6.91</v>
+        <v>4.85</v>
       </c>
       <c r="L4" t="n">
-        <v>1866.62</v>
+        <v>967.64</v>
       </c>
       <c r="M4" t="n">
-        <v>0.24</v>
+        <v>0.27</v>
       </c>
       <c r="N4" t="n">
-        <v>2799.92</v>
+        <v>1451.45</v>
       </c>
       <c r="O4" t="n">
-        <v>6.5</v>
+        <v>6.45</v>
       </c>
       <c r="P4" t="n">
-        <v>157.82</v>
+        <v>67.64</v>
       </c>
       <c r="Q4" t="n">
         <v>10</v>
       </c>
       <c r="R4" t="n">
-        <v>5.36</v>
+        <v>-7.87</v>
       </c>
       <c r="S4" t="n">
-        <v>5.36</v>
+        <v>-7.86</v>
       </c>
       <c r="T4" t="n">
-        <v>19.78</v>
+        <v>16.79</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>92</v>
+        <v>61</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>WIPRO</t>
+          <t>VARUNBEV</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>WIPRO India Limited</t>
+          <t>VARUNBEV India Limited</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Oil &amp; Gas</t>
+          <t>Power</t>
         </is>
       </c>
       <c r="E5" t="n">
-        <v>54.71</v>
+        <v>43.49</v>
       </c>
       <c r="F5" t="n">
-        <v>44.95</v>
+        <v>19.9</v>
       </c>
       <c r="G5" t="n">
-        <v>56.78</v>
+        <v>27.36</v>
       </c>
       <c r="H5" t="n">
-        <v>16.16</v>
+        <v>11.87</v>
       </c>
       <c r="I5" s="2" t="n">
         <v>0.4</v>
       </c>
       <c r="J5" t="n">
-        <v>9.51</v>
+        <v>7.61</v>
       </c>
       <c r="L5" t="n">
-        <v>1930.88</v>
+        <v>1470.72</v>
       </c>
       <c r="M5" t="n">
-        <v>0.36</v>
+        <v>0.64</v>
       </c>
       <c r="N5" t="n">
-        <v>2896.32</v>
+        <v>2206.08</v>
       </c>
       <c r="O5" t="n">
-        <v>8.619999999999999</v>
+        <v>14.25</v>
       </c>
       <c r="P5" t="n">
-        <v>136.39</v>
+        <v>58.84</v>
       </c>
       <c r="Q5" t="n">
         <v>10</v>
       </c>
       <c r="R5" t="n">
-        <v>15.37</v>
+        <v>14.28</v>
       </c>
       <c r="S5" t="n">
-        <v>15.37</v>
+        <v>14.28</v>
       </c>
       <c r="T5" t="n">
-        <v>15.05</v>
+        <v>17.17</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>VEDL</t>
+          <t>RECLTD</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>VEDL India Limited</t>
+          <t>RECLTD India Limited</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>IT</t>
+          <t>Construction</t>
         </is>
       </c>
       <c r="E6" t="n">
-        <v>50.81</v>
+        <v>39.6</v>
       </c>
       <c r="F6" t="n">
-        <v>56.18</v>
+        <v>27.41</v>
       </c>
       <c r="G6" t="n">
-        <v>73.8</v>
+        <v>40.89</v>
       </c>
       <c r="H6" t="n">
-        <v>13.95</v>
+        <v>9.289999999999999</v>
       </c>
       <c r="I6" s="2" t="n">
         <v>0.4</v>
       </c>
       <c r="J6" t="n">
-        <v>8.529999999999999</v>
+        <v>6.46</v>
       </c>
       <c r="L6" t="n">
-        <v>1540.87</v>
+        <v>1742.94</v>
       </c>
       <c r="M6" t="n">
-        <v>0.68</v>
+        <v>0.34</v>
       </c>
       <c r="N6" t="n">
-        <v>2311.31</v>
+        <v>2614.41</v>
       </c>
       <c r="O6" t="n">
-        <v>12.54</v>
+        <v>10.77</v>
       </c>
       <c r="P6" t="n">
-        <v>72.66</v>
+        <v>86.45</v>
       </c>
       <c r="Q6" t="n">
         <v>10</v>
       </c>
       <c r="R6" t="n">
-        <v>5.61</v>
+        <v>12.75</v>
       </c>
       <c r="S6" t="n">
-        <v>5.61</v>
+        <v>12.75</v>
       </c>
       <c r="T6" t="n">
-        <v>19.69</v>
+        <v>21.49</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>28</v>
+        <v>32</v>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>M_M</t>
+          <t>SIEMENS</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>M_M India Limited</t>
+          <t>SIEMENS India Limited</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>IT</t>
+          <t>Metals</t>
         </is>
       </c>
       <c r="E7" t="n">
-        <v>49.79</v>
+        <v>38.2</v>
       </c>
       <c r="F7" t="n">
-        <v>60.33</v>
+        <v>27.01</v>
       </c>
       <c r="G7" t="n">
-        <v>78.64</v>
+        <v>37.47</v>
       </c>
       <c r="H7" t="n">
-        <v>14.28</v>
+        <v>11.53</v>
       </c>
       <c r="I7" s="2" t="n">
         <v>0.4</v>
       </c>
       <c r="J7" t="n">
-        <v>8.68</v>
+        <v>7.46</v>
       </c>
       <c r="L7" t="n">
-        <v>1639.42</v>
+        <v>1267.58</v>
       </c>
       <c r="M7" t="n">
-        <v>0.18</v>
+        <v>0.47</v>
       </c>
       <c r="N7" t="n">
-        <v>2459.12</v>
+        <v>1901.37</v>
       </c>
       <c r="O7" t="n">
-        <v>4.36</v>
+        <v>8.24</v>
       </c>
       <c r="P7" t="n">
-        <v>223.31</v>
+        <v>87.03</v>
       </c>
       <c r="Q7" t="n">
         <v>10</v>
       </c>
       <c r="R7" t="n">
-        <v>12.38</v>
+        <v>9.9</v>
       </c>
       <c r="S7" t="n">
-        <v>12.38</v>
+        <v>9.9</v>
       </c>
       <c r="T7" t="n">
-        <v>20.65</v>
+        <v>20.58</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>31</v>
+        <v>39</v>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>ADANIPORTS</t>
+          <t>INDUSINDBK</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>ADANIPORTS India Limited</t>
+          <t>INDUSINDBK India Limited</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Automobile</t>
+          <t>Consumer Goods</t>
         </is>
       </c>
       <c r="E8" t="n">
-        <v>48.38</v>
+        <v>37.07</v>
       </c>
       <c r="F8" t="n">
-        <v>80.73999999999999</v>
+        <v>33.17</v>
       </c>
       <c r="G8" t="n">
-        <v>101.04</v>
+        <v>44.53</v>
       </c>
       <c r="H8" t="n">
-        <v>16.79</v>
+        <v>12.85</v>
       </c>
       <c r="I8" s="2" t="n">
         <v>0.4</v>
       </c>
       <c r="J8" t="n">
-        <v>9.800000000000001</v>
+        <v>8.039999999999999</v>
       </c>
       <c r="L8" t="n">
-        <v>683.89</v>
+        <v>695.16</v>
       </c>
       <c r="M8" t="n">
-        <v>0.31</v>
+        <v>0.35</v>
       </c>
       <c r="N8" t="n">
-        <v>1025.83</v>
+        <v>1042.75</v>
       </c>
       <c r="O8" t="n">
-        <v>1.81</v>
+        <v>3.23</v>
       </c>
       <c r="P8" t="n">
-        <v>231.72</v>
+        <v>124.76</v>
       </c>
       <c r="Q8" t="n">
         <v>10</v>
       </c>
       <c r="R8" t="n">
-        <v>32.29</v>
+        <v>19.91</v>
       </c>
       <c r="S8" t="n">
-        <v>32.29</v>
+        <v>19.91</v>
       </c>
       <c r="T8" t="n">
-        <v>17.81</v>
+        <v>18.45</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
-        <v>6</v>
+        <v>13</v>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>BHARTIARTL</t>
+          <t>HCLTECH</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>BHARTIARTL India Limited</t>
+          <t>HCLTECH India Limited</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Pharma</t>
+          <t>Automobile</t>
         </is>
       </c>
       <c r="E9" t="n">
-        <v>42.59</v>
+        <v>31.17</v>
       </c>
       <c r="F9" t="n">
-        <v>53.5</v>
+        <v>53.73</v>
       </c>
       <c r="G9" t="n">
-        <v>75.53</v>
+        <v>80.19</v>
       </c>
       <c r="H9" t="n">
-        <v>10.92</v>
+        <v>9.32</v>
       </c>
       <c r="I9" s="2" t="n">
         <v>0.4</v>
       </c>
       <c r="J9" t="n">
-        <v>7.19</v>
+        <v>6.47</v>
       </c>
       <c r="L9" t="n">
-        <v>1489.79</v>
+        <v>554.6799999999999</v>
       </c>
       <c r="M9" t="n">
-        <v>0.18</v>
+        <v>0.36</v>
       </c>
       <c r="N9" t="n">
-        <v>2234.68</v>
+        <v>832.03</v>
       </c>
       <c r="O9" t="n">
-        <v>5.84</v>
+        <v>4.53</v>
       </c>
       <c r="P9" t="n">
-        <v>142.52</v>
+        <v>65.44</v>
       </c>
       <c r="Q9" t="n">
         <v>10</v>
       </c>
       <c r="R9" t="n">
-        <v>14.38</v>
+        <v>12.97</v>
       </c>
       <c r="S9" t="n">
-        <v>14.38</v>
+        <v>12.97</v>
       </c>
       <c r="T9" t="n">
-        <v>18.21</v>
+        <v>19.02</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
-        <v>38</v>
+        <v>79</v>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>VBL</t>
+          <t>IDFCFIRSTB</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>VBL India Limited</t>
+          <t>IDFCFIRSTB India Limited</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Oil &amp; Gas</t>
+          <t>Power</t>
         </is>
       </c>
       <c r="E10" t="n">
-        <v>37.81</v>
+        <v>22.17</v>
       </c>
       <c r="F10" t="n">
-        <v>32.62</v>
+        <v>23.15</v>
       </c>
       <c r="G10" t="n">
-        <v>48.43</v>
+        <v>39.94</v>
       </c>
       <c r="H10" t="n">
-        <v>9.43</v>
+        <v>6.48</v>
       </c>
       <c r="I10" s="2" t="n">
         <v>0.4</v>
       </c>
       <c r="J10" t="n">
-        <v>6.52</v>
+        <v>5.21</v>
       </c>
       <c r="L10" t="n">
-        <v>1577.06</v>
+        <v>1173.45</v>
       </c>
       <c r="M10" t="n">
-        <v>0.34</v>
+        <v>0.3</v>
       </c>
       <c r="N10" t="n">
-        <v>2365.59</v>
+        <v>1760.18</v>
       </c>
       <c r="O10" t="n">
-        <v>11.23</v>
+        <v>7.61</v>
       </c>
       <c r="P10" t="n">
-        <v>75.37</v>
+        <v>73.29000000000001</v>
       </c>
       <c r="Q10" t="n">
         <v>10</v>
       </c>
       <c r="R10" t="n">
-        <v>9.93</v>
+        <v>-2.34</v>
       </c>
       <c r="S10" t="n">
-        <v>9.93</v>
+        <v>-2.33</v>
       </c>
       <c r="T10" t="n">
-        <v>17.07</v>
+        <v>18.84</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>MARUTI</t>
+          <t>SUNPHARMA</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>MARUTI India Limited</t>
+          <t>SUNPHARMA India Limited</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Metals</t>
+          <t>Pharma</t>
         </is>
       </c>
       <c r="E11" t="n">
-        <v>36.94</v>
+        <v>16.39</v>
       </c>
       <c r="F11" t="n">
-        <v>23.13</v>
+        <v>18.14</v>
       </c>
       <c r="G11" t="n">
-        <v>38.19</v>
+        <v>28.06</v>
       </c>
       <c r="H11" t="n">
-        <v>7.18</v>
+        <v>8.43</v>
       </c>
       <c r="I11" s="2" t="n">
         <v>0.4</v>
       </c>
       <c r="J11" t="n">
-        <v>5.52</v>
+        <v>6.08</v>
       </c>
       <c r="L11" t="n">
-        <v>1747.25</v>
+        <v>540.23</v>
       </c>
       <c r="M11" t="n">
-        <v>0.88</v>
+        <v>0.23</v>
       </c>
       <c r="N11" t="n">
-        <v>2620.88</v>
+        <v>810.34</v>
       </c>
       <c r="O11" t="n">
-        <v>16.77</v>
+        <v>3.25</v>
       </c>
       <c r="P11" t="n">
-        <v>51.33</v>
+        <v>86.41</v>
       </c>
       <c r="Q11" t="n">
         <v>10</v>
       </c>
       <c r="R11" t="n">
-        <v>-1.59</v>
+        <v>-2.54</v>
       </c>
       <c r="S11" t="n">
-        <v>-1.59</v>
+        <v>-2.54</v>
       </c>
       <c r="T11" t="n">
-        <v>20.76</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="n">
-        <v>42</v>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>GODREJCP</t>
-        </is>
-      </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>GODREJCP India Limited</t>
-        </is>
-      </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>Pharma</t>
-        </is>
-      </c>
-      <c r="E12" t="n">
-        <v>32.34</v>
-      </c>
-      <c r="F12" t="n">
-        <v>34.42</v>
-      </c>
-      <c r="G12" t="n">
-        <v>53.61</v>
-      </c>
-      <c r="H12" t="n">
-        <v>8.279999999999999</v>
-      </c>
-      <c r="I12" s="2" t="n">
-        <v>0.4</v>
-      </c>
-      <c r="J12" t="n">
-        <v>6.01</v>
-      </c>
-      <c r="L12" t="n">
-        <v>1615.04</v>
-      </c>
-      <c r="M12" t="n">
-        <v>0.24</v>
-      </c>
-      <c r="N12" t="n">
-        <v>2422.55</v>
-      </c>
-      <c r="O12" t="n">
-        <v>6.28</v>
-      </c>
-      <c r="P12" t="n">
-        <v>132.75</v>
-      </c>
-      <c r="Q12" t="n">
-        <v>10</v>
-      </c>
-      <c r="R12" t="n">
-        <v>1.03</v>
-      </c>
-      <c r="S12" t="n">
-        <v>1.03</v>
-      </c>
-      <c r="T12" t="n">
-        <v>19.67</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="n">
-        <v>3</v>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>HDFCBANK</t>
-        </is>
-      </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>HDFCBANK India Limited</t>
-        </is>
-      </c>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t>Consumer Goods</t>
-        </is>
-      </c>
-      <c r="E13" t="n">
-        <v>26.79</v>
-      </c>
-      <c r="F13" t="n">
-        <v>19.55</v>
-      </c>
-      <c r="G13" t="n">
-        <v>30.34</v>
-      </c>
-      <c r="H13" t="n">
-        <v>8.359999999999999</v>
-      </c>
-      <c r="I13" s="2" t="n">
-        <v>0.4</v>
-      </c>
-      <c r="J13" t="n">
-        <v>6.05</v>
-      </c>
-      <c r="L13" t="n">
-        <v>1007.66</v>
-      </c>
-      <c r="M13" t="n">
-        <v>0.43</v>
-      </c>
-      <c r="N13" t="n">
-        <v>1511.48</v>
-      </c>
-      <c r="O13" t="n">
-        <v>5.59</v>
-      </c>
-      <c r="P13" t="n">
-        <v>93.28</v>
-      </c>
-      <c r="Q13" t="n">
-        <v>10</v>
-      </c>
-      <c r="R13" t="n">
-        <v>5.03</v>
-      </c>
-      <c r="S13" t="n">
-        <v>5.03</v>
-      </c>
-      <c r="T13" t="n">
-        <v>17.11</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="n">
-        <v>2</v>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>TCS</t>
-        </is>
-      </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>TCS India Limited</t>
-        </is>
-      </c>
-      <c r="D14" t="inlineStr">
-        <is>
-          <t>Oil &amp; Gas</t>
-        </is>
-      </c>
-      <c r="E14" t="n">
-        <v>22.16</v>
-      </c>
-      <c r="F14" t="n">
-        <v>17.21</v>
-      </c>
-      <c r="G14" t="n">
-        <v>31.27</v>
-      </c>
-      <c r="H14" t="n">
-        <v>5.81</v>
-      </c>
-      <c r="I14" s="2" t="n">
-        <v>0.4</v>
-      </c>
-      <c r="J14" t="n">
-        <v>4.91</v>
-      </c>
-      <c r="L14" t="n">
-        <v>986.34</v>
-      </c>
-      <c r="M14" t="n">
-        <v>0.63</v>
-      </c>
-      <c r="N14" t="n">
-        <v>1479.51</v>
-      </c>
-      <c r="O14" t="n">
-        <v>16.92</v>
-      </c>
-      <c r="P14" t="n">
-        <v>26.56</v>
-      </c>
-      <c r="Q14" t="n">
-        <v>10</v>
-      </c>
-      <c r="R14" t="n">
-        <v>-2.71</v>
-      </c>
-      <c r="S14" t="n">
-        <v>-2.71</v>
-      </c>
-      <c r="T14" t="n">
-        <v>18.74</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="n">
-        <v>36</v>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>IOC</t>
-        </is>
-      </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>IOC India Limited</t>
-        </is>
-      </c>
-      <c r="D15" t="inlineStr">
-        <is>
-          <t>Financial Services</t>
-        </is>
-      </c>
-      <c r="E15" t="n">
-        <v>21.09</v>
-      </c>
-      <c r="F15" t="n">
-        <v>18.35</v>
-      </c>
-      <c r="G15" t="n">
-        <v>31</v>
-      </c>
-      <c r="H15" t="n">
-        <v>6.8</v>
-      </c>
-      <c r="I15" s="2" t="n">
-        <v>0.4</v>
-      </c>
-      <c r="J15" t="n">
-        <v>5.36</v>
-      </c>
-      <c r="L15" t="n">
-        <v>1169.56</v>
-      </c>
-      <c r="M15" t="n">
-        <v>0.34</v>
-      </c>
-      <c r="N15" t="n">
-        <v>1754.33</v>
-      </c>
-      <c r="O15" t="n">
-        <v>9.23</v>
-      </c>
-      <c r="P15" t="n">
-        <v>61.27</v>
-      </c>
-      <c r="Q15" t="n">
-        <v>10</v>
-      </c>
-      <c r="R15" t="n">
-        <v>-5.42</v>
-      </c>
-      <c r="S15" t="n">
-        <v>-5.42</v>
-      </c>
-      <c r="T15" t="n">
-        <v>15.47</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="n">
-        <v>15</v>
-      </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>SUNPHARMA</t>
-        </is>
-      </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>SUNPHARMA India Limited</t>
-        </is>
-      </c>
-      <c r="D16" t="inlineStr">
-        <is>
-          <t>Pharma</t>
-        </is>
-      </c>
-      <c r="E16" t="n">
-        <v>16.39</v>
-      </c>
-      <c r="F16" t="n">
-        <v>18.14</v>
-      </c>
-      <c r="G16" t="n">
-        <v>28.06</v>
-      </c>
-      <c r="H16" t="n">
-        <v>8.43</v>
-      </c>
-      <c r="I16" s="2" t="n">
-        <v>0.4</v>
-      </c>
-      <c r="J16" t="n">
-        <v>6.08</v>
-      </c>
-      <c r="L16" t="n">
-        <v>540.23</v>
-      </c>
-      <c r="M16" t="n">
-        <v>0.23</v>
-      </c>
-      <c r="N16" t="n">
-        <v>810.34</v>
-      </c>
-      <c r="O16" t="n">
-        <v>3.25</v>
-      </c>
-      <c r="P16" t="n">
-        <v>86.41</v>
-      </c>
-      <c r="Q16" t="n">
-        <v>10</v>
-      </c>
-      <c r="R16" t="n">
-        <v>-2.54</v>
-      </c>
-      <c r="S16" t="n">
-        <v>-2.54</v>
-      </c>
-      <c r="T16" t="n">
-        <v>20.03</v>
+        <v>20.55</v>
       </c>
     </row>
   </sheetData>
@@ -2339,7 +2014,7 @@
         <v>28.43</v>
       </c>
       <c r="T2" t="n">
-        <v>15.39</v>
+        <v>18.01</v>
       </c>
     </row>
     <row r="3">
@@ -2404,7 +2079,7 @@
         <v>24.76</v>
       </c>
       <c r="T3" t="n">
-        <v>29.3</v>
+        <v>18.56</v>
       </c>
     </row>
     <row r="4">
@@ -2469,7 +2144,7 @@
         <v>20.61</v>
       </c>
       <c r="T4" t="n">
-        <v>32.99</v>
+        <v>31.27</v>
       </c>
     </row>
     <row r="5">
@@ -2534,7 +2209,7 @@
         <v>26.28</v>
       </c>
       <c r="T5" t="n">
-        <v>18.61</v>
+        <v>32.66</v>
       </c>
     </row>
     <row r="6">
@@ -2599,7 +2274,7 @@
         <v>16.36</v>
       </c>
       <c r="T6" t="n">
-        <v>33.72</v>
+        <v>17.28</v>
       </c>
     </row>
     <row r="7">
@@ -2664,7 +2339,7 @@
         <v>12.99</v>
       </c>
       <c r="T7" t="n">
-        <v>16.03</v>
+        <v>34.66</v>
       </c>
     </row>
     <row r="8">
@@ -2729,7 +2404,7 @@
         <v>15.24</v>
       </c>
       <c r="T8" t="n">
-        <v>34.15</v>
+        <v>33.92</v>
       </c>
     </row>
     <row r="9">
@@ -2794,7 +2469,7 @@
         <v>31.76</v>
       </c>
       <c r="T9" t="n">
-        <v>19.6</v>
+        <v>29.51</v>
       </c>
     </row>
     <row r="10">
@@ -2859,7 +2534,7 @@
         <v>13.31</v>
       </c>
       <c r="T10" t="n">
-        <v>15.12</v>
+        <v>22.92</v>
       </c>
     </row>
     <row r="11">
@@ -2924,7 +2599,7 @@
         <v>17.78</v>
       </c>
       <c r="T11" t="n">
-        <v>17.76</v>
+        <v>33.18</v>
       </c>
     </row>
     <row r="12">
@@ -2989,7 +2664,7 @@
         <v>21.6</v>
       </c>
       <c r="T12" t="n">
-        <v>29.15</v>
+        <v>24.02</v>
       </c>
     </row>
     <row r="13">
@@ -3054,7 +2729,7 @@
         <v>15.37</v>
       </c>
       <c r="T13" t="n">
-        <v>15.05</v>
+        <v>30.72</v>
       </c>
     </row>
     <row r="14">
@@ -3119,7 +2794,7 @@
         <v>25.43</v>
       </c>
       <c r="T14" t="n">
-        <v>16.69</v>
+        <v>17.69</v>
       </c>
     </row>
     <row r="15">
@@ -3184,7 +2859,7 @@
         <v>19.06</v>
       </c>
       <c r="T15" t="n">
-        <v>23.2</v>
+        <v>32.53</v>
       </c>
     </row>
     <row r="16">
@@ -3249,7 +2924,7 @@
         <v>23.71</v>
       </c>
       <c r="T16" t="n">
-        <v>28.28</v>
+        <v>28.99</v>
       </c>
     </row>
     <row r="17">
@@ -3314,7 +2989,7 @@
         <v>13.36</v>
       </c>
       <c r="T17" t="n">
-        <v>29.5</v>
+        <v>22.81</v>
       </c>
     </row>
     <row r="18">
@@ -3379,7 +3054,7 @@
         <v>14.29</v>
       </c>
       <c r="T18" t="n">
-        <v>16.47</v>
+        <v>17.79</v>
       </c>
     </row>
     <row r="19">
@@ -3444,7 +3119,7 @@
         <v>12.38</v>
       </c>
       <c r="T19" t="n">
-        <v>20.65</v>
+        <v>24.24</v>
       </c>
     </row>
     <row r="20">
@@ -3509,7 +3184,7 @@
         <v>13.59</v>
       </c>
       <c r="T20" t="n">
-        <v>26.65</v>
+        <v>34.75</v>
       </c>
     </row>
     <row r="21">
@@ -3574,7 +3249,7 @@
         <v>32.29</v>
       </c>
       <c r="T21" t="n">
-        <v>17.81</v>
+        <v>27.8</v>
       </c>
     </row>
     <row r="22">
@@ -3639,7 +3314,7 @@
         <v>18.59</v>
       </c>
       <c r="T22" t="n">
-        <v>27.43</v>
+        <v>31.45</v>
       </c>
     </row>
     <row r="23">
@@ -3704,7 +3379,7 @@
         <v>22.78</v>
       </c>
       <c r="T23" t="n">
-        <v>26.4</v>
+        <v>34.76</v>
       </c>
     </row>
     <row r="24">
@@ -3769,7 +3444,7 @@
         <v>17.2</v>
       </c>
       <c r="T24" t="n">
-        <v>34.08</v>
+        <v>30.28</v>
       </c>
     </row>
     <row r="25">
@@ -3834,7 +3509,7 @@
         <v>14.28</v>
       </c>
       <c r="T25" t="n">
-        <v>28.95</v>
+        <v>17.17</v>
       </c>
     </row>
     <row r="26">
@@ -3899,7 +3574,7 @@
         <v>14.38</v>
       </c>
       <c r="T26" t="n">
-        <v>18.21</v>
+        <v>21.49</v>
       </c>
     </row>
     <row r="27">
@@ -3964,7 +3639,7 @@
         <v>13.25</v>
       </c>
       <c r="T27" t="n">
-        <v>30.17</v>
+        <v>33.59</v>
       </c>
     </row>
     <row r="28">
@@ -4029,7 +3704,7 @@
         <v>12.75</v>
       </c>
       <c r="T28" t="n">
-        <v>34.52</v>
+        <v>21.49</v>
       </c>
     </row>
     <row r="29">
@@ -4094,7 +3769,7 @@
         <v>20.25</v>
       </c>
       <c r="T29" t="n">
-        <v>29.49</v>
+        <v>18.97</v>
       </c>
     </row>
     <row r="30">
@@ -4159,7 +3834,7 @@
         <v>19.91</v>
       </c>
       <c r="T30" t="n">
-        <v>16.79</v>
+        <v>18.45</v>
       </c>
     </row>
     <row r="31">
@@ -4224,7 +3899,7 @@
         <v>12.97</v>
       </c>
       <c r="T31" t="n">
-        <v>34.87</v>
+        <v>19.02</v>
       </c>
     </row>
     <row r="32">
@@ -4289,7 +3964,7 @@
         <v>21.18</v>
       </c>
       <c r="T32" t="n">
-        <v>26.37</v>
+        <v>27.17</v>
       </c>
     </row>
     <row r="33">
@@ -4354,7 +4029,7 @@
         <v>13.6</v>
       </c>
       <c r="T33" t="n">
-        <v>27.12</v>
+        <v>17.83</v>
       </c>
     </row>
   </sheetData>
@@ -4535,7 +4210,7 @@
         <v>28.43</v>
       </c>
       <c r="T2" t="n">
-        <v>15.39</v>
+        <v>18.01</v>
       </c>
     </row>
     <row r="3">
@@ -4600,7 +4275,7 @@
         <v>24.76</v>
       </c>
       <c r="T3" t="n">
-        <v>29.3</v>
+        <v>18.56</v>
       </c>
     </row>
     <row r="4">
@@ -4665,7 +4340,7 @@
         <v>20.61</v>
       </c>
       <c r="T4" t="n">
-        <v>32.99</v>
+        <v>31.27</v>
       </c>
     </row>
     <row r="5">
@@ -4730,7 +4405,7 @@
         <v>26.28</v>
       </c>
       <c r="T5" t="n">
-        <v>18.61</v>
+        <v>32.66</v>
       </c>
     </row>
     <row r="6">
@@ -4795,7 +4470,7 @@
         <v>16.36</v>
       </c>
       <c r="T6" t="n">
-        <v>33.72</v>
+        <v>17.28</v>
       </c>
     </row>
     <row r="7">
@@ -4860,7 +4535,7 @@
         <v>12.99</v>
       </c>
       <c r="T7" t="n">
-        <v>16.03</v>
+        <v>34.66</v>
       </c>
     </row>
     <row r="8">
@@ -4925,7 +4600,7 @@
         <v>15.24</v>
       </c>
       <c r="T8" t="n">
-        <v>34.15</v>
+        <v>33.92</v>
       </c>
     </row>
     <row r="9">
@@ -4990,7 +4665,7 @@
         <v>31.76</v>
       </c>
       <c r="T9" t="n">
-        <v>19.6</v>
+        <v>29.51</v>
       </c>
     </row>
     <row r="10">
@@ -5055,7 +4730,7 @@
         <v>13.31</v>
       </c>
       <c r="T10" t="n">
-        <v>15.12</v>
+        <v>22.92</v>
       </c>
     </row>
     <row r="11">
@@ -5120,7 +4795,7 @@
         <v>17.78</v>
       </c>
       <c r="T11" t="n">
-        <v>17.76</v>
+        <v>33.18</v>
       </c>
     </row>
     <row r="12">
@@ -5185,7 +4860,7 @@
         <v>21.6</v>
       </c>
       <c r="T12" t="n">
-        <v>29.15</v>
+        <v>24.02</v>
       </c>
     </row>
     <row r="13">
@@ -5250,7 +4925,7 @@
         <v>5.36</v>
       </c>
       <c r="T13" t="n">
-        <v>19.78</v>
+        <v>29.18</v>
       </c>
     </row>
     <row r="14">
@@ -5315,7 +4990,7 @@
         <v>15.37</v>
       </c>
       <c r="T14" t="n">
-        <v>15.05</v>
+        <v>30.72</v>
       </c>
     </row>
     <row r="15">
@@ -5380,7 +5055,7 @@
         <v>8.48</v>
       </c>
       <c r="T15" t="n">
-        <v>25.83</v>
+        <v>32.89</v>
       </c>
     </row>
     <row r="16">
@@ -5445,7 +5120,7 @@
         <v>25.43</v>
       </c>
       <c r="T16" t="n">
-        <v>16.69</v>
+        <v>17.69</v>
       </c>
     </row>
     <row r="17">
@@ -5510,7 +5185,7 @@
         <v>19.06</v>
       </c>
       <c r="T17" t="n">
-        <v>23.2</v>
+        <v>32.53</v>
       </c>
     </row>
     <row r="18">
@@ -5575,7 +5250,7 @@
         <v>-5.95</v>
       </c>
       <c r="T18" t="n">
-        <v>26.97</v>
+        <v>25.08</v>
       </c>
     </row>
     <row r="19">
@@ -5640,7 +5315,7 @@
         <v>23.71</v>
       </c>
       <c r="T19" t="n">
-        <v>28.28</v>
+        <v>28.99</v>
       </c>
     </row>
     <row r="20">
@@ -5705,7 +5380,7 @@
         <v>13.36</v>
       </c>
       <c r="T20" t="n">
-        <v>29.5</v>
+        <v>22.81</v>
       </c>
     </row>
     <row r="21">
@@ -5770,7 +5445,7 @@
         <v>5.61</v>
       </c>
       <c r="T21" t="n">
-        <v>19.69</v>
+        <v>27.88</v>
       </c>
     </row>
     <row r="22">
@@ -5835,7 +5510,7 @@
         <v>14.29</v>
       </c>
       <c r="T22" t="n">
-        <v>16.47</v>
+        <v>17.79</v>
       </c>
     </row>
     <row r="23">
@@ -5900,7 +5575,7 @@
         <v>12.38</v>
       </c>
       <c r="T23" t="n">
-        <v>20.65</v>
+        <v>24.24</v>
       </c>
     </row>
     <row r="24">
@@ -5965,7 +5640,7 @@
         <v>1.8</v>
       </c>
       <c r="T24" t="n">
-        <v>24.11</v>
+        <v>17.9</v>
       </c>
     </row>
     <row r="25">
@@ -6030,7 +5705,7 @@
         <v>13.59</v>
       </c>
       <c r="T25" t="n">
-        <v>26.65</v>
+        <v>34.75</v>
       </c>
     </row>
     <row r="26">
@@ -6095,7 +5770,7 @@
         <v>32.29</v>
       </c>
       <c r="T26" t="n">
-        <v>17.81</v>
+        <v>27.8</v>
       </c>
     </row>
     <row r="27">
@@ -6160,7 +5835,7 @@
         <v>18.59</v>
       </c>
       <c r="T27" t="n">
-        <v>27.43</v>
+        <v>31.45</v>
       </c>
     </row>
     <row r="28">
@@ -6225,7 +5900,7 @@
         <v>22.78</v>
       </c>
       <c r="T28" t="n">
-        <v>26.4</v>
+        <v>34.76</v>
       </c>
     </row>
     <row r="29">
@@ -6290,7 +5965,7 @@
         <v>-7.86</v>
       </c>
       <c r="T29" t="n">
-        <v>33.09</v>
+        <v>16.79</v>
       </c>
     </row>
     <row r="30">
@@ -6355,7 +6030,7 @@
         <v>5.44</v>
       </c>
       <c r="T30" t="n">
-        <v>23.39</v>
+        <v>20.73</v>
       </c>
     </row>
     <row r="31">
@@ -6420,7 +6095,7 @@
         <v>3.48</v>
       </c>
       <c r="T31" t="n">
-        <v>25.15</v>
+        <v>23.67</v>
       </c>
     </row>
     <row r="32">
@@ -6485,7 +6160,7 @@
         <v>9.359999999999999</v>
       </c>
       <c r="T32" t="n">
-        <v>30.68</v>
+        <v>34.74</v>
       </c>
     </row>
     <row r="33">
@@ -6550,7 +6225,7 @@
         <v>17.2</v>
       </c>
       <c r="T33" t="n">
-        <v>34.08</v>
+        <v>30.28</v>
       </c>
     </row>
     <row r="34">
@@ -6615,7 +6290,7 @@
         <v>7.06</v>
       </c>
       <c r="T34" t="n">
-        <v>33.25</v>
+        <v>27.47</v>
       </c>
     </row>
     <row r="35">
@@ -6680,7 +6355,7 @@
         <v>9.41</v>
       </c>
       <c r="T35" t="n">
-        <v>29.07</v>
+        <v>22.23</v>
       </c>
     </row>
     <row r="36">
@@ -6745,7 +6420,7 @@
         <v>14.28</v>
       </c>
       <c r="T36" t="n">
-        <v>28.95</v>
+        <v>17.17</v>
       </c>
     </row>
     <row r="37">
@@ -6810,7 +6485,7 @@
         <v>11.67</v>
       </c>
       <c r="T37" t="n">
-        <v>20.03</v>
+        <v>32.99</v>
       </c>
     </row>
     <row r="38">
@@ -6875,7 +6550,7 @@
         <v>10.78</v>
       </c>
       <c r="T38" t="n">
-        <v>30.98</v>
+        <v>26.78</v>
       </c>
     </row>
     <row r="39">
@@ -6940,7 +6615,7 @@
         <v>11.84</v>
       </c>
       <c r="T39" t="n">
-        <v>17.94</v>
+        <v>29.79</v>
       </c>
     </row>
     <row r="40">
@@ -7005,7 +6680,7 @@
         <v>14.38</v>
       </c>
       <c r="T40" t="n">
-        <v>18.21</v>
+        <v>21.49</v>
       </c>
     </row>
     <row r="41">
@@ -7070,7 +6745,7 @@
         <v>13.25</v>
       </c>
       <c r="T41" t="n">
-        <v>30.17</v>
+        <v>33.59</v>
       </c>
     </row>
     <row r="42">
@@ -7135,7 +6810,7 @@
         <v>0.47</v>
       </c>
       <c r="T42" t="n">
-        <v>17.92</v>
+        <v>32.82</v>
       </c>
     </row>
     <row r="43">
@@ -7200,7 +6875,7 @@
         <v>-2.73</v>
       </c>
       <c r="T43" t="n">
-        <v>20.7</v>
+        <v>15.95</v>
       </c>
     </row>
     <row r="44">
@@ -7265,7 +6940,7 @@
         <v>0.04</v>
       </c>
       <c r="T44" t="n">
-        <v>26.84</v>
+        <v>26.89</v>
       </c>
     </row>
     <row r="45">
@@ -7330,7 +7005,7 @@
         <v>12.75</v>
       </c>
       <c r="T45" t="n">
-        <v>34.52</v>
+        <v>21.49</v>
       </c>
     </row>
     <row r="46">
@@ -7395,7 +7070,7 @@
         <v>5.81</v>
       </c>
       <c r="T46" t="n">
-        <v>20.58</v>
+        <v>23.01</v>
       </c>
     </row>
     <row r="47">
@@ -7460,7 +7135,7 @@
         <v>5.29</v>
       </c>
       <c r="T47" t="n">
-        <v>20.72</v>
+        <v>18.54</v>
       </c>
     </row>
     <row r="48">
@@ -7525,7 +7200,7 @@
         <v>9.9</v>
       </c>
       <c r="T48" t="n">
-        <v>19.48</v>
+        <v>20.58</v>
       </c>
     </row>
     <row r="49">
@@ -7590,7 +7265,7 @@
         <v>10.08</v>
       </c>
       <c r="T49" t="n">
-        <v>21.44</v>
+        <v>28.4</v>
       </c>
     </row>
     <row r="50">
@@ -7655,7 +7330,7 @@
         <v>9.93</v>
       </c>
       <c r="T50" t="n">
-        <v>17.07</v>
+        <v>25.1</v>
       </c>
     </row>
     <row r="51">
@@ -7720,7 +7395,7 @@
         <v>20.25</v>
       </c>
       <c r="T51" t="n">
-        <v>29.49</v>
+        <v>18.97</v>
       </c>
     </row>
     <row r="52">
@@ -7785,7 +7460,7 @@
         <v>-2.79</v>
       </c>
       <c r="T52" t="n">
-        <v>24.95</v>
+        <v>22.14</v>
       </c>
     </row>
     <row r="53">
@@ -7850,7 +7525,7 @@
         <v>9.81</v>
       </c>
       <c r="T53" t="n">
-        <v>34.67</v>
+        <v>30.67</v>
       </c>
     </row>
     <row r="54">
@@ -7915,7 +7590,7 @@
         <v>19.91</v>
       </c>
       <c r="T54" t="n">
-        <v>16.79</v>
+        <v>18.45</v>
       </c>
     </row>
     <row r="55">
@@ -7980,7 +7655,7 @@
         <v>9.960000000000001</v>
       </c>
       <c r="T55" t="n">
-        <v>31.51</v>
+        <v>20.38</v>
       </c>
     </row>
     <row r="56">
@@ -8045,7 +7720,7 @@
         <v>-1.59</v>
       </c>
       <c r="T56" t="n">
-        <v>20.76</v>
+        <v>20.13</v>
       </c>
     </row>
     <row r="57">
@@ -8110,7 +7785,7 @@
         <v>11.32</v>
       </c>
       <c r="T57" t="n">
-        <v>18.13</v>
+        <v>26.24</v>
       </c>
     </row>
     <row r="58">
@@ -8175,7 +7850,7 @@
         <v>8.16</v>
       </c>
       <c r="T58" t="n">
-        <v>33.31</v>
+        <v>25.32</v>
       </c>
     </row>
     <row r="59">
@@ -8240,7 +7915,7 @@
         <v>-3.74</v>
       </c>
       <c r="T59" t="n">
-        <v>21.26</v>
+        <v>25.6</v>
       </c>
     </row>
     <row r="60">
@@ -8305,7 +7980,7 @@
         <v>-9.15</v>
       </c>
       <c r="T60" t="n">
-        <v>25.16</v>
+        <v>29.88</v>
       </c>
     </row>
     <row r="61">
@@ -8370,7 +8045,7 @@
         <v>0.45</v>
       </c>
       <c r="T61" t="n">
-        <v>34.35</v>
+        <v>33.35</v>
       </c>
     </row>
     <row r="62">
@@ -8435,7 +8110,7 @@
         <v>-8.140000000000001</v>
       </c>
       <c r="T62" t="n">
-        <v>21.06</v>
+        <v>24.87</v>
       </c>
     </row>
     <row r="63">
@@ -8500,7 +8175,7 @@
         <v>5.37</v>
       </c>
       <c r="T63" t="n">
-        <v>32.39</v>
+        <v>34.89</v>
       </c>
     </row>
     <row r="64">
@@ -8565,7 +8240,7 @@
         <v>-10.41</v>
       </c>
       <c r="T64" t="n">
-        <v>18.01</v>
+        <v>30.69</v>
       </c>
     </row>
     <row r="65">
@@ -8630,7 +8305,7 @@
         <v>1.03</v>
       </c>
       <c r="T65" t="n">
-        <v>19.67</v>
+        <v>31.29</v>
       </c>
     </row>
     <row r="66">
@@ -8695,7 +8370,7 @@
         <v>8</v>
       </c>
       <c r="T66" t="n">
-        <v>33.49</v>
+        <v>23.74</v>
       </c>
     </row>
     <row r="67">
@@ -8760,7 +8435,7 @@
         <v>12.97</v>
       </c>
       <c r="T67" t="n">
-        <v>34.87</v>
+        <v>19.02</v>
       </c>
     </row>
     <row r="68">
@@ -8825,7 +8500,7 @@
         <v>21.18</v>
       </c>
       <c r="T68" t="n">
-        <v>26.37</v>
+        <v>27.17</v>
       </c>
     </row>
     <row r="69">
@@ -8890,7 +8565,7 @@
         <v>2.52</v>
       </c>
       <c r="T69" t="n">
-        <v>31.6</v>
+        <v>32.06</v>
       </c>
     </row>
     <row r="70">
@@ -8955,7 +8630,7 @@
         <v>-7.65</v>
       </c>
       <c r="T70" t="n">
-        <v>22.85</v>
+        <v>30.66</v>
       </c>
     </row>
     <row r="71">
@@ -9020,7 +8695,7 @@
         <v>8.33</v>
       </c>
       <c r="T71" t="n">
-        <v>19.89</v>
+        <v>30.1</v>
       </c>
     </row>
     <row r="72">
@@ -9085,7 +8760,7 @@
         <v>-2.58</v>
       </c>
       <c r="T72" t="n">
-        <v>34.2</v>
+        <v>26.25</v>
       </c>
     </row>
     <row r="73">
@@ -9150,7 +8825,7 @@
         <v>0.57</v>
       </c>
       <c r="T73" t="n">
-        <v>28.07</v>
+        <v>24.79</v>
       </c>
     </row>
     <row r="74">
@@ -9215,7 +8890,7 @@
         <v>-3.07</v>
       </c>
       <c r="T74" t="n">
-        <v>25.4</v>
+        <v>33.53</v>
       </c>
     </row>
     <row r="75">
@@ -9280,7 +8955,7 @@
         <v>13.6</v>
       </c>
       <c r="T75" t="n">
-        <v>27.12</v>
+        <v>17.83</v>
       </c>
     </row>
     <row r="76">
@@ -9345,7 +9020,7 @@
         <v>5.03</v>
       </c>
       <c r="T76" t="n">
-        <v>17.11</v>
+        <v>25.26</v>
       </c>
     </row>
     <row r="77">
@@ -9410,7 +9085,7 @@
         <v>-4.55</v>
       </c>
       <c r="T77" t="n">
-        <v>16.02</v>
+        <v>16.05</v>
       </c>
     </row>
     <row r="78">
@@ -9475,7 +9150,7 @@
         <v>1.96</v>
       </c>
       <c r="T78" t="n">
-        <v>29.11</v>
+        <v>26.72</v>
       </c>
     </row>
     <row r="79">
@@ -9540,7 +9215,7 @@
         <v>-11.8</v>
       </c>
       <c r="T79" t="n">
-        <v>25.86</v>
+        <v>23.85</v>
       </c>
     </row>
     <row r="80">
@@ -9605,7 +9280,7 @@
         <v>5.67</v>
       </c>
       <c r="T80" t="n">
-        <v>19.06</v>
+        <v>28.92</v>
       </c>
     </row>
     <row r="81">
@@ -9670,7 +9345,7 @@
         <v>-11.01</v>
       </c>
       <c r="T81" t="n">
-        <v>24.9</v>
+        <v>30.65</v>
       </c>
     </row>
     <row r="82">
@@ -9735,7 +9410,7 @@
         <v>-11.93</v>
       </c>
       <c r="T82" t="n">
-        <v>15.4</v>
+        <v>25.09</v>
       </c>
     </row>
     <row r="83">
@@ -9800,7 +9475,7 @@
         <v>-2.18</v>
       </c>
       <c r="T83" t="n">
-        <v>31.74</v>
+        <v>34.52</v>
       </c>
     </row>
     <row r="84">
@@ -9865,7 +9540,7 @@
         <v>8.68</v>
       </c>
       <c r="T84" t="n">
-        <v>24.96</v>
+        <v>25.37</v>
       </c>
     </row>
     <row r="85">
@@ -9930,7 +9605,7 @@
         <v>-2.33</v>
       </c>
       <c r="T85" t="n">
-        <v>31.34</v>
+        <v>18.84</v>
       </c>
     </row>
     <row r="86">
@@ -9995,7 +9670,7 @@
         <v>-2.71</v>
       </c>
       <c r="T86" t="n">
-        <v>18.74</v>
+        <v>32.5</v>
       </c>
     </row>
     <row r="87">
@@ -10060,7 +9735,7 @@
         <v>-5.29</v>
       </c>
       <c r="T87" t="n">
-        <v>23.39</v>
+        <v>16.71</v>
       </c>
     </row>
     <row r="88">
@@ -10125,7 +9800,7 @@
         <v>-5.42</v>
       </c>
       <c r="T88" t="n">
-        <v>15.47</v>
+        <v>23.47</v>
       </c>
     </row>
     <row r="89">
@@ -10190,7 +9865,7 @@
         <v>-5.41</v>
       </c>
       <c r="T89" t="n">
-        <v>31.41</v>
+        <v>30.19</v>
       </c>
     </row>
     <row r="90">
@@ -10255,7 +9930,7 @@
         <v>-6.13</v>
       </c>
       <c r="T90" t="n">
-        <v>30.25</v>
+        <v>24.7</v>
       </c>
     </row>
     <row r="91">
@@ -10320,7 +9995,7 @@
         <v>4.44</v>
       </c>
       <c r="T91" t="n">
-        <v>23.08</v>
+        <v>34.35</v>
       </c>
     </row>
     <row r="92">
@@ -10385,7 +10060,7 @@
         <v>-7.85</v>
       </c>
       <c r="T92" t="n">
-        <v>22.04</v>
+        <v>31.03</v>
       </c>
     </row>
     <row r="93">
@@ -10450,7 +10125,7 @@
         <v>-2.54</v>
       </c>
       <c r="T93" t="n">
-        <v>20.03</v>
+        <v>20.55</v>
       </c>
     </row>
   </sheetData>
@@ -10631,7 +10306,7 @@
         <v>13.59</v>
       </c>
       <c r="T2" t="n">
-        <v>26.65</v>
+        <v>34.75</v>
       </c>
     </row>
     <row r="3">
@@ -10696,7 +10371,7 @@
         <v>18.59</v>
       </c>
       <c r="T3" t="n">
-        <v>27.43</v>
+        <v>31.45</v>
       </c>
     </row>
     <row r="4">
@@ -10761,7 +10436,7 @@
         <v>22.78</v>
       </c>
       <c r="T4" t="n">
-        <v>26.4</v>
+        <v>34.76</v>
       </c>
     </row>
     <row r="5">
@@ -10826,7 +10501,7 @@
         <v>9.41</v>
       </c>
       <c r="T5" t="n">
-        <v>29.07</v>
+        <v>22.23</v>
       </c>
     </row>
     <row r="6">
@@ -10891,7 +10566,7 @@
         <v>0.47</v>
       </c>
       <c r="T6" t="n">
-        <v>17.92</v>
+        <v>32.82</v>
       </c>
     </row>
     <row r="7">
@@ -10956,7 +10631,7 @@
         <v>0.57</v>
       </c>
       <c r="T7" t="n">
-        <v>28.07</v>
+        <v>24.79</v>
       </c>
     </row>
     <row r="8">
@@ -11021,7 +10696,7 @@
         <v>-2.18</v>
       </c>
       <c r="T8" t="n">
-        <v>31.74</v>
+        <v>34.52</v>
       </c>
     </row>
     <row r="9">
@@ -11086,7 +10761,7 @@
         <v>-5.42</v>
       </c>
       <c r="T9" t="n">
-        <v>15.47</v>
+        <v>23.47</v>
       </c>
     </row>
   </sheetData>
@@ -11267,7 +10942,7 @@
         <v>13.59</v>
       </c>
       <c r="T2" t="n">
-        <v>26.65</v>
+        <v>34.75</v>
       </c>
     </row>
     <row r="3">
@@ -11332,7 +11007,7 @@
         <v>18.59</v>
       </c>
       <c r="T3" t="n">
-        <v>27.43</v>
+        <v>31.45</v>
       </c>
     </row>
     <row r="4">
@@ -11397,7 +11072,7 @@
         <v>22.78</v>
       </c>
       <c r="T4" t="n">
-        <v>26.4</v>
+        <v>34.76</v>
       </c>
     </row>
     <row r="5">
@@ -11462,7 +11137,7 @@
         <v>9.41</v>
       </c>
       <c r="T5" t="n">
-        <v>29.07</v>
+        <v>22.23</v>
       </c>
     </row>
     <row r="6">
@@ -11527,7 +11202,7 @@
         <v>0.47</v>
       </c>
       <c r="T6" t="n">
-        <v>17.92</v>
+        <v>32.82</v>
       </c>
     </row>
     <row r="7">
@@ -11592,7 +11267,7 @@
         <v>0.45</v>
       </c>
       <c r="T7" t="n">
-        <v>34.35</v>
+        <v>33.35</v>
       </c>
     </row>
     <row r="8">
@@ -11657,7 +11332,7 @@
         <v>0.57</v>
       </c>
       <c r="T8" t="n">
-        <v>28.07</v>
+        <v>24.79</v>
       </c>
     </row>
     <row r="9">
@@ -11722,7 +11397,7 @@
         <v>-11.8</v>
       </c>
       <c r="T9" t="n">
-        <v>25.86</v>
+        <v>23.85</v>
       </c>
     </row>
     <row r="10">
@@ -11787,7 +11462,7 @@
         <v>-2.18</v>
       </c>
       <c r="T10" t="n">
-        <v>31.74</v>
+        <v>34.52</v>
       </c>
     </row>
     <row r="11">
@@ -11852,7 +11527,7 @@
         <v>-5.42</v>
       </c>
       <c r="T11" t="n">
-        <v>15.47</v>
+        <v>23.47</v>
       </c>
     </row>
   </sheetData>

</xml_diff>